<commit_message>
Rebuild murl_dashboard.xlsx with single-spill architecture
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel/murl_dashboard.xlsx
+++ b/Excel/murl_dashboard.xlsx
@@ -22,15 +22,12 @@
     <definedName name="f_requester">Dashboard!$D$11</definedName>
     <definedName name="f_status">Dashboard!$A$11</definedName>
     <definedName name="f_target">Dashboard!$G$9</definedName>
-    <definedName name="f_topn">Dashboard!$D$22</definedName>
     <definedName name="lstActivation">Lists!$I$1:$I$1</definedName>
     <definedName name="lstDivision">Lists!$G$1:$G$1</definedName>
     <definedName name="lstRegion">Lists!$E$1:$E$1</definedName>
     <definedName name="lstRequester">Lists!$C$1:$C$1</definedName>
     <definedName name="lstStatus">Lists!$A$1:$A$1</definedName>
-    <definedName name="lstTopN">Lists!$K$1:$K$4</definedName>
     <definedName name="rngFilter">Dashboard!$A$24#</definedName>
-    <definedName name="rngFilterFull">Lists!$P$1#</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="52">
   <si>
     <t>Labels</t>
   </si>
@@ -67,7 +64,7 @@
     <t>Reference</t>
   </si>
   <si>
-    <t>Summary</t>
+    <t>MURL</t>
   </si>
   <si>
     <t>Service project</t>
@@ -88,7 +85,7 @@
     <t>Line manager</t>
   </si>
   <si>
-    <t>MURL Name</t>
+    <t>MURL name</t>
   </si>
   <si>
     <t>Activation</t>
@@ -106,10 +103,7 @@
     <t>Business Division requested for</t>
   </si>
   <si>
-    <t>Target Default</t>
-  </si>
-  <si>
-    <t>Alle</t>
+    <t>Target URL</t>
   </si>
   <si>
     <t>MURL Dashboard</t>
@@ -167,9 +161,6 @@
   </si>
   <si>
     <t>ERGEBNISSE</t>
-  </si>
-  <si>
-    <t>Anzeigen:</t>
   </si>
   <si>
     <t>Anleitung — MURL Dashboard (Pro)</t>
@@ -575,20 +566,20 @@
   <tableColumns count="16">
     <tableColumn id="1" name="Labels"/>
     <tableColumn id="2" name="Reference"/>
-    <tableColumn id="3" name="Summary"/>
+    <tableColumn id="3" name="MURL"/>
     <tableColumn id="4" name="Service project"/>
     <tableColumn id="5" name="Status"/>
     <tableColumn id="6" name="Requester"/>
     <tableColumn id="7" name="Type"/>
     <tableColumn id="8" name="Region(s)"/>
     <tableColumn id="9" name="Line manager"/>
-    <tableColumn id="10" name="MURL Name"/>
+    <tableColumn id="10" name="MURL name"/>
     <tableColumn id="11" name="Activation"/>
     <tableColumn id="12" name="Properties"/>
     <tableColumn id="13" name="GOTO/MURL Owner 1"/>
     <tableColumn id="14" name="GOTO/MURL Owner 2"/>
     <tableColumn id="15" name="Business Division requested for"/>
-    <tableColumn id="16" name="Target Default"/>
+    <tableColumn id="16" name="Target URL"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -898,7 +889,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="40" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -918,7 +909,7 @@
     </row>
     <row r="2" spans="1:16" ht="22" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -938,58 +929,58 @@
     </row>
     <row r="4" spans="1:16" ht="22" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="J4" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
       <c r="M4" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
     </row>
     <row r="5" spans="1:16" ht="44" customHeight="1">
       <c r="A5" s="8">
-        <f>IFERROR(IF(COLUMNS(rngFilterFull)&gt;1,ROWS(rngFilterFull),0),0)</f>
+        <f>IFERROR(IF(COLUMNS(rngFilter)&gt;1,ROWS(rngFilter),0),0)</f>
         <v>0</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8">
-        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilterFull,0,5)="Active")),0)</f>
+        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilter,0,5)="Active")),0)</f>
         <v>0</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8">
-        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilterFull,0,5)="Scheduled Activation")),0)</f>
+        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilter,0,5)="Scheduled Activation")),0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8">
-        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilterFull,0,5)="Pending Change")),0)</f>
+        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilter,0,5)="Pending Change")),0)</f>
         <v>0</v>
       </c>
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
       <c r="M5" s="8">
-        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilterFull,0,5)="Deactivated")),0)</f>
+        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilter,0,5)="Deactivated")),0)</f>
         <v>0</v>
       </c>
       <c r="N5" s="8"/>
@@ -997,27 +988,27 @@
     </row>
     <row r="7" spans="1:16" ht="22" customHeight="1">
       <c r="A7" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="18" customHeight="1">
       <c r="A8" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
       <c r="G8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
       <c r="J8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K8" s="10"/>
       <c r="L8" s="10"/>
@@ -1048,12 +1039,12 @@
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="G10" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
       <c r="J10" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K10" s="10"/>
       <c r="L10" s="10"/>
@@ -1082,7 +1073,7 @@
     </row>
     <row r="13" spans="1:16" ht="22" customHeight="1">
       <c r="A13" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="24" customHeight="1">
@@ -1093,19 +1084,19 @@
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="E14" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J14" s="12"/>
       <c r="K14" s="12"/>
       <c r="L14" s="12"/>
       <c r="M14" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
@@ -1113,77 +1104,77 @@
     </row>
     <row r="15" spans="1:16" ht="20" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
       <c r="D15" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J15" s="13"/>
       <c r="K15" s="13"/>
       <c r="L15" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N15" s="13"/>
       <c r="O15" s="13"/>
       <c r="P15" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="20" customHeight="1">
       <c r="A16" s="15" cm="1">
-        <f t="array" ref="A16">IFERROR(LET(col,LET(c,INDEX(rngFilterFull,0,5),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
+        <f t="array" ref="A16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,5),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
         <v>0</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="16" cm="1">
-        <f t="array" ref="D16">IFERROR(LET(col,LET(c,INDEX(rngFilterFull,0,5),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
+        <f t="array" ref="D16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,5),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
         <v>0</v>
       </c>
       <c r="E16" s="15" cm="1">
-        <f t="array" ref="E16">IFERROR(LET(col,LET(c,INDEX(rngFilterFull,0,15),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
+        <f t="array" ref="E16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,15),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
         <v>0</v>
       </c>
       <c r="F16" s="15"/>
       <c r="G16" s="15"/>
       <c r="H16" s="16" cm="1">
-        <f t="array" ref="H16">IFERROR(LET(col,LET(c,INDEX(rngFilterFull,0,15),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
+        <f t="array" ref="H16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,15),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
         <v>0</v>
       </c>
       <c r="I16" s="15" cm="1">
-        <f t="array" ref="I16">IFERROR(LET(col,LET(c,INDEX(rngFilterFull,0,8),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
+        <f t="array" ref="I16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,8),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
         <v>0</v>
       </c>
       <c r="J16" s="15"/>
       <c r="K16" s="15"/>
       <c r="L16" s="16" cm="1">
-        <f t="array" ref="L16">IFERROR(LET(col,LET(c,INDEX(rngFilterFull,0,8),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
+        <f t="array" ref="L16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,8),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
         <v>0</v>
       </c>
       <c r="M16" s="15" cm="1">
-        <f t="array" ref="M16">IFERROR(LET(col,LET(c1,INDEX(rngFilterFull,0,13),c2,INDEX(rngFilterFull,0,14),IFERROR(_xlfn._xlws.FILTER(_xlfn.VSTACK(c1,c2),_xlfn.VSTACK(c1,c2)&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
+        <f t="array" ref="M16">IFERROR(LET(col,LET(c1,INDEX(rngFilter,0,13),c2,INDEX(rngFilter,0,14),IFERROR(_xlfn._xlws.FILTER(_xlfn.VSTACK(c1,c2),_xlfn.VSTACK(c1,c2)&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
         <v>0</v>
       </c>
       <c r="N16" s="15"/>
       <c r="O16" s="15"/>
       <c r="P16" s="16" cm="1">
-        <f t="array" ref="P16">IFERROR(LET(col,LET(c1,INDEX(rngFilterFull,0,13),c2,INDEX(rngFilterFull,0,14),IFERROR(_xlfn._xlws.FILTER(_xlfn.VSTACK(c1,c2),_xlfn.VSTACK(c1,c2)&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
+        <f t="array" ref="P16">IFERROR(LET(col,LET(c1,INDEX(rngFilter,0,13),c2,INDEX(rngFilter,0,14),IFERROR(_xlfn._xlws.FILTER(_xlfn.VSTACK(c1,c2),_xlfn.VSTACK(c1,c2)&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
         <v>0</v>
       </c>
     </row>
@@ -1261,13 +1252,7 @@
     </row>
     <row r="22" spans="1:16" ht="24" customHeight="1">
       <c r="A22" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="F22" s="17">
         <f>IF((f_labels&lt;&gt;"")+(f_murl&lt;&gt;"")+(f_target&lt;&gt;"")+(f_owner&lt;&gt;"")+(f_status&lt;&gt;"")+(f_requester&lt;&gt;"")+(f_region&lt;&gt;"")+(f_division&lt;&gt;"")+(f_activation&lt;&gt;"")&gt;0,"FILTER AKTIV","Keine Filter gesetzt")</f>
@@ -1276,7 +1261,7 @@
       <c r="G22" s="17"/>
       <c r="H22" s="17"/>
       <c r="K22" s="18">
-        <f>"Zeigt " &amp; IF(COLUMNS(rngFilterFull)&gt;1,TEXT(ROWS(rngFilterFull),"#'##0"),0) &amp; " von " &amp; TEXT(ROWS(tblData),"#'##0") &amp; " Einträgen"</f>
+        <f>"Zeigt " &amp; IF(COLUMNS(rngFilter)&gt;1,TEXT(ROWS(rngFilter),"#'##0"),0) &amp; " von " &amp; TEXT(ROWS(tblData),"#'##0") &amp; " Einträgen"</f>
         <v>0</v>
       </c>
       <c r="L22" s="18"/>
@@ -1337,7 +1322,7 @@
     </row>
     <row r="24" spans="1:16">
       <c r="A24" cm="1">
-        <f t="array" ref="A24">LET(f,IFERROR(_xlfn._xlws.FILTER(tblData,(tblData[Reference]&lt;&gt;"")*((f_labels="")+ISNUMBER(SEARCH(f_labels,tblData[Labels])))*((f_murl="")+ISNUMBER(SEARCH(f_murl,tblData[MURL Name])))*((f_target="")+ISNUMBER(SEARCH(f_target,tblData[Target Default])))*((f_owner="")+ISNUMBER(SEARCH(f_owner,tblData[GOTO/MURL Owner 1]))+ISNUMBER(SEARCH(f_owner,tblData[GOTO/MURL Owner 2])))*((f_status="")+ISNUMBER(SEARCH(f_status,tblData[Status])))*((f_requester="")+ISNUMBER(SEARCH(f_requester,tblData[Requester])))*((f_region="")+ISNUMBER(SEARCH(f_region,tblData[Region(s)])))*((f_division="")+ISNUMBER(SEARCH(f_division,tblData[Business Division requested for])))*((f_activation="")+ISNUMBER(SEARCH(f_activation,tblData[Activation])))),"Keine Treffer — Filter zurücksetzen"),IF(ISNUMBER(f_topn),IFERROR(_xlfn.TAKE(f,f_topn),f),f))</f>
+        <f t="array" ref="A24">IFERROR(_xlfn._xlws.FILTER(tblData,(tblData[Reference]&lt;&gt;"")*((f_labels="")+ISNUMBER(SEARCH(f_labels,tblData[Labels])))*((f_murl="")+ISNUMBER(SEARCH(f_murl,tblData[MURL name])))*((f_target="")+ISNUMBER(SEARCH(f_target,tblData[Target URL])))*((f_owner="")+ISNUMBER(SEARCH(f_owner,tblData[GOTO/MURL Owner 1]))+ISNUMBER(SEARCH(f_owner,tblData[GOTO/MURL Owner 2])))*((f_status="")+ISNUMBER(SEARCH(f_status,tblData[Status])))*((f_requester="")+ISNUMBER(SEARCH(f_requester,tblData[Requester])))*((f_region="")+ISNUMBER(SEARCH(f_region,tblData[Region(s)])))*((f_division="")+ISNUMBER(SEARCH(f_division,tblData[Business Division requested for])))*((f_activation="")+ISNUMBER(SEARCH(f_activation,tblData[Activation])))),"Keine Treffer — Filter zurücksetzen")</f>
         <v>0</v>
       </c>
     </row>
@@ -1404,7 +1389,7 @@
     <mergeCell ref="F22:H22"/>
     <mergeCell ref="K22:P22"/>
   </mergeCells>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="A11">
       <formula1>Lists!$A$1:$A$1</formula1>
     </dataValidation>
@@ -1419,9 +1404,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="M11">
       <formula1>Lists!$I$1:$I$1</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="D22">
-      <formula1>Lists!$K$1:$K$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1507,34 +1489,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="K1:P4"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="11:16">
-      <c r="K1">
-        <v>50</v>
-      </c>
-      <c r="P1" cm="1">
-        <f t="array" ref="P1">IFERROR(_xlfn._xlws.FILTER(tblData,(tblData[Reference]&lt;&gt;"")*((f_labels="")+ISNUMBER(SEARCH(f_labels,tblData[Labels])))*((f_murl="")+ISNUMBER(SEARCH(f_murl,tblData[MURL Name])))*((f_target="")+ISNUMBER(SEARCH(f_target,tblData[Target Default])))*((f_owner="")+ISNUMBER(SEARCH(f_owner,tblData[GOTO/MURL Owner 1]))+ISNUMBER(SEARCH(f_owner,tblData[GOTO/MURL Owner 2])))*((f_status="")+ISNUMBER(SEARCH(f_status,tblData[Status])))*((f_requester="")+ISNUMBER(SEARCH(f_requester,tblData[Requester])))*((f_region="")+ISNUMBER(SEARCH(f_region,tblData[Region(s)])))*((f_division="")+ISNUMBER(SEARCH(f_division,tblData[Business Division requested for])))*((f_activation="")+ISNUMBER(SEARCH(f_activation,tblData[Activation])))),"Keine Treffer — Filter zurücksetzen")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="11:16">
-      <c r="K2">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="3" spans="11:16">
-      <c r="K3">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="4" spans="11:16">
-      <c r="K4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1549,7 +1506,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="32" customHeight="1">
       <c r="A1" s="20" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -1557,27 +1514,27 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="22" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="21" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:1">
@@ -1585,12 +1542,12 @@
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:1">
@@ -1598,32 +1555,32 @@
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="21" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:1">
@@ -1631,17 +1588,17 @@
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="21" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use static range for rngFilter instead of spill anchor
Some Excel for Windows 365 builds strip named ranges that reference a spill
anchor (#), even though it's officially supported. Replace =Dashboard!\$A\$24#
with the static range =Dashboard!\$A\$24:\$P\$30000 and update the two
formulas that depended on ROWS(rngFilter) reflecting the spill size — they
now count non-empty Reference cells via SUMPRODUCT.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel/murl_dashboard.xlsx
+++ b/Excel/murl_dashboard.xlsx
@@ -27,7 +27,7 @@
     <definedName name="lstRegion">Lists!$E$1:$E$1</definedName>
     <definedName name="lstRequester">Lists!$C$1:$C$1</definedName>
     <definedName name="lstStatus">Lists!$A$1:$A$1</definedName>
-    <definedName name="rngFilter">Dashboard!$A$24#</definedName>
+    <definedName name="rngFilter">Dashboard!$A$24:$P$30000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -956,7 +956,7 @@
     </row>
     <row r="5" spans="1:16" ht="44" customHeight="1">
       <c r="A5" s="8">
-        <f>IFERROR(IF(COLUMNS(rngFilter)&gt;1,ROWS(rngFilter),0),0)</f>
+        <f>IFERROR(SUMPRODUCT(--(INDEX(rngFilter,0,2)&lt;&gt;"")),0)</f>
         <v>0</v>
       </c>
       <c r="B5" s="8"/>
@@ -1261,7 +1261,7 @@
       <c r="G22" s="17"/>
       <c r="H22" s="17"/>
       <c r="K22" s="18">
-        <f>"Zeigt " &amp; IF(COLUMNS(rngFilter)&gt;1,TEXT(ROWS(rngFilter),"#'##0"),0) &amp; " von " &amp; TEXT(ROWS(tblData),"#'##0") &amp; " Einträgen"</f>
+        <f>"Zeigt " &amp; TEXT(SUMPRODUCT(--(INDEX(rngFilter,0,2)&lt;&gt;"")),"#'##0") &amp; " von " &amp; TEXT(ROWS(tblData),"#'##0") &amp; " Einträgen"</f>
         <v>0</v>
       </c>
       <c r="L22" s="18"/>

</xml_diff>

<commit_message>
Remove mini-pivot aggregations to avoid LAMBDA/TAKE compatibility issues
The 8 mini-pivot formulas chained LAMBDA, BYROW, CHOOSECOLS and TAKE —
all 2022-era Excel 365 additions. Corp Windows Excel on Semi-Annual
Channel rejects these and strips the formulas on file open, triggering
the repair dialog. Drop the AGGREGATION section entirely; the remaining
dashboard (KPIs + filters + filter-active indicator + hit counter +
results spill) uses only widely-supported functions.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel/murl_dashboard.xlsx
+++ b/Excel/murl_dashboard.xlsx
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
     <t>Labels</t>
   </si>
@@ -146,18 +146,6 @@
   </si>
   <si>
     <t>Business Division</t>
-  </si>
-  <si>
-    <t>AGGREGATION — Top 5 im aktuellen Filter</t>
-  </si>
-  <si>
-    <t>Wert</t>
-  </si>
-  <si>
-    <t>Anzahl</t>
-  </si>
-  <si>
-    <t>Top Owners</t>
   </si>
   <si>
     <t>ERGEBNISSE</t>
@@ -218,7 +206,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,29 +269,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF404040"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFE60000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -319,8 +284,23 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="18"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF404040"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -360,7 +340,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -470,20 +450,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFCCCABC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -518,37 +489,22 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1071,252 +1027,73 @@
       <c r="N11" s="11"/>
       <c r="O11" s="11"/>
     </row>
-    <row r="13" spans="1:16" ht="22" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="24" customHeight="1">
-      <c r="A14" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="12"/>
-    </row>
-    <row r="15" spans="1:16" ht="20" customHeight="1">
-      <c r="A15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="M15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="20" customHeight="1">
-      <c r="A16" s="15" cm="1">
-        <f t="array" ref="A16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,5),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16" cm="1">
-        <f t="array" ref="D16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,5),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="15" cm="1">
-        <f t="array" ref="E16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,15),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16" cm="1">
-        <f t="array" ref="H16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,15),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="I16" s="15" cm="1">
-        <f t="array" ref="I16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,8),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="16" cm="1">
-        <f t="array" ref="L16">IFERROR(LET(col,LET(c,INDEX(rngFilter,0,8),IFERROR(_xlfn._xlws.FILTER(c,c&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="15" cm="1">
-        <f t="array" ref="M16">IFERROR(LET(col,LET(c1,INDEX(rngFilter,0,13),c2,INDEX(rngFilter,0,14),IFERROR(_xlfn._xlws.FILTER(_xlfn.VSTACK(c1,c2),_xlfn.VSTACK(c1,c2)&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),1)),"")</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="16" cm="1">
-        <f t="array" ref="P16">IFERROR(LET(col,LET(c1,INDEX(rngFilter,0,13),c2,INDEX(rngFilter,0,14),IFERROR(_xlfn._xlws.FILTER(_xlfn.VSTACK(c1,c2),_xlfn.VSTACK(c1,c2)&lt;&gt;""),"")),u,IFERROR(_xlfn.UNIQUE(col),""),c,IFERROR(_xlfn.BYROW(u,_xlfn.LAMBDA(v,SUMPRODUCT(--(col=v)))),0),_xlfn.CHOOSECOLS(_xlfn.TAKE(_xlfn._xlws.SORT(_xlfn.HSTACK(u,c),2,-1),5),2)),"")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="20" customHeight="1">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="15"/>
-      <c r="N17" s="15"/>
-      <c r="O17" s="15"/>
-      <c r="P17" s="16"/>
-    </row>
-    <row r="18" spans="1:16" ht="20" customHeight="1">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="16"/>
-    </row>
-    <row r="19" spans="1:16" ht="20" customHeight="1">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="15"/>
-      <c r="N19" s="15"/>
-      <c r="O19" s="15"/>
-      <c r="P19" s="16"/>
-    </row>
-    <row r="20" spans="1:16" ht="20" customHeight="1">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="16"/>
-    </row>
     <row r="22" spans="1:16" ht="24" customHeight="1">
       <c r="A22" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F22" s="17">
+        <v>30</v>
+      </c>
+      <c r="F22" s="12">
         <f>IF((f_labels&lt;&gt;"")+(f_murl&lt;&gt;"")+(f_target&lt;&gt;"")+(f_owner&lt;&gt;"")+(f_status&lt;&gt;"")+(f_requester&lt;&gt;"")+(f_region&lt;&gt;"")+(f_division&lt;&gt;"")+(f_activation&lt;&gt;"")&gt;0,"FILTER AKTIV","Keine Filter gesetzt")</f>
         <v>0</v>
       </c>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="K22" s="18">
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="K22" s="13">
         <f>"Zeigt " &amp; TEXT(SUMPRODUCT(--(INDEX(rngFilter,0,2)&lt;&gt;"")),"#,##0") &amp; " von " &amp; TEXT(ROWS(tblData),"#,##0") &amp; " Einträgen"</f>
         <v>0</v>
       </c>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="18"/>
-      <c r="P22" s="18"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
     </row>
     <row r="23" spans="1:16" ht="26" customHeight="1">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H23" s="19" t="s">
+      <c r="H23" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I23" s="19" t="s">
+      <c r="I23" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J23" s="19" t="s">
+      <c r="J23" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K23" s="19" t="s">
+      <c r="K23" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L23" s="19" t="s">
+      <c r="L23" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="M23" s="19" t="s">
+      <c r="M23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="N23" s="19" t="s">
+      <c r="N23" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="O23" s="19" t="s">
+      <c r="O23" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="P23" s="19" t="s">
+      <c r="P23" s="14" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1327,7 +1104,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="32">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A4:C4"/>
@@ -1358,34 +1135,6 @@
     <mergeCell ref="J11:L11"/>
     <mergeCell ref="M10:O10"/>
     <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="I14:L14"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="M14:P14"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="M18:O18"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:O20"/>
     <mergeCell ref="F22:H22"/>
     <mergeCell ref="K22:P22"/>
   </mergeCells>
@@ -1505,100 +1254,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="32" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="16"/>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="21"/>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="22" t="s">
+    <row r="7" spans="1:1">
+      <c r="A7" s="16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="21" t="s">
+    <row r="8" spans="1:1">
+      <c r="A8" s="16"/>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="17" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="21" t="s">
+    <row r="10" spans="1:1">
+      <c r="A10" s="16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="21" t="s">
+    <row r="11" spans="1:1">
+      <c r="A11" s="16"/>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="17" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="21" t="s">
+    <row r="13" spans="1:1">
+      <c r="A13" s="16" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="21"/>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="22" t="s">
+    <row r="14" spans="1:1">
+      <c r="A14" s="16" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="21"/>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="21" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" s="21" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="16"/>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="16" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="21" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" s="16" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" s="21" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" s="21"/>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="22" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="21" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="21" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>